<commit_message>
Moved book 'Matar a un ruiseñor' from wishlist to biblioteca
</commit_message>
<xml_diff>
--- a/data/nini/Wishlist.xlsx
+++ b/data/nini/Wishlist.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -773,54 +773,50 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Matar a un ruiseñor</t>
+          <t>La M de las moscas</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Harper Lee</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Lumen</t>
-        </is>
-      </c>
+          <t>Helena Araújo</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>La M de las moscas</t>
+          <t>Siddhartha</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Helena Araújo</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
+          <t>Herman Hesse</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Debolsillo Edición Especial en Tapa Dura</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Siddhartha</t>
+          <t>Afrodita</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Herman Hesse</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Debolsillo Edición Especial en Tapa Dura</t>
-        </is>
-      </c>
+          <t>Isabel Allende</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Afrodita</t>
+          <t xml:space="preserve">Amor </t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -833,7 +829,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Amor </t>
+          <t>Cuentos de Eva Luna</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -846,7 +842,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cuentos de Eva Luna</t>
+          <t>El juego de Ripper</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -859,7 +855,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>El juego de Ripper</t>
+          <t>El plan infinito</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -872,7 +868,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>El plan infinito</t>
+          <t>El viento conoce mi nombre</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -885,7 +881,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>El viento conoce mi nombre</t>
+          <t>El Zorro: comienza la leyenda</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -898,7 +894,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>El Zorro: comienza la leyenda</t>
+          <t>Inés del alma mía</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -911,7 +907,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Inés del alma mía</t>
+          <t>La gorda de porcelana</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -924,7 +920,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>La gorda de porcelana</t>
+          <t>Largo pétalo de mar</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -937,7 +933,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Largo pétalo de mar</t>
+          <t>Los amantes del Guggenheim</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -950,7 +946,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Los amantes del Guggenheim</t>
+          <t>Mi país inventado</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -963,7 +959,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mi país inventado</t>
+          <t>Mujeres del alma mía</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -976,7 +972,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mujeres del alma mía</t>
+          <t>Paula</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -989,12 +985,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Paula</t>
+          <t>El señor de los anillos</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Isabel Allende</t>
+          <t>J.R.R. Tolkien</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1002,12 +998,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>El señor de los anillos</t>
+          <t>Juvenilia</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>J.R.R. Tolkien</t>
+          <t>Jane Austen</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1015,12 +1011,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Juvenilia</t>
+          <t>El principio del mundo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Jane Austen</t>
+          <t>Jeremías Gamboa</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1028,12 +1024,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>El principio del mundo</t>
+          <t>Los viejos marineros</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jeremías Gamboa</t>
+          <t>Jorge Amador</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -1041,25 +1037,29 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Los viejos marineros</t>
+          <t>El Aleph</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Jorge Amador</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
+          <t>Jorge Luis Borges</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Debolsillo Edición Especial en Tapa Dura</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>El Aleph</t>
+          <t>Ensayo sobre la ceguera</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jorge Luis Borges</t>
+          <t>José Saramago</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1071,29 +1071,25 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Ensayo sobre la ceguera</t>
+          <t>Tú no matarás</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>José Saramago</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Debolsillo Edición Especial en Tapa Dura</t>
-        </is>
-      </c>
+          <t>Julia Navarro</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tú no matarás</t>
+          <t>Pan piedra</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Julia Navarro</t>
+          <t>Laura Andrea Garzón</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -1101,12 +1097,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Pan piedra</t>
+          <t>Delirio</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Laura Andrea Garzón</t>
+          <t>Laura Restrepo</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -1114,7 +1110,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Delirio</t>
+          <t>Los Divinos</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1127,12 +1123,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Los Divinos</t>
+          <t>Una noche en el paraíso</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Laura Restrepo</t>
+          <t>Lucía Berlín</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -1140,12 +1136,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Una noche en el paraíso</t>
+          <t>Las amazonas: mito e historia</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Lucía Berlín</t>
+          <t>Lyn Webster Wild</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -1153,12 +1149,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Las amazonas: mito e historia</t>
+          <t>Hamnet</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Lyn Webster Wild</t>
+          <t>Maggie O'Farrell</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -1166,12 +1162,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Hamnet</t>
+          <t>Chambacú, corral de negros</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Maggie O'Farrell</t>
+          <t>Manuel Zapata Olivella</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -1179,7 +1175,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chambacú, corral de negros</t>
+          <t>Changó, el gran putas</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1192,7 +1188,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Changó, el gran putas</t>
+          <t>En Chimá nace un santo</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1205,12 +1201,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>En Chimá nace un santo</t>
+          <t>El sonido de las olas</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Manuel Zapata Olivella</t>
+          <t>Margarita García Robayo</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -1218,7 +1214,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>El sonido de las olas</t>
+          <t>Primera persona</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1231,12 +1227,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Primera persona</t>
+          <t>Al otro lado del Mar</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Margarita García Robayo</t>
+          <t>María Cristina Restrepo</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -1244,12 +1240,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Al otro lado del Mar</t>
+          <t>Lais</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>María Cristina Restrepo</t>
+          <t>María de Francia</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -1257,12 +1253,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Lais</t>
+          <t>Cartas a un joven sicólogo</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>María de Francia</t>
+          <t>María Dolores Avia</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -1270,12 +1266,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Cartas a un joven sicólogo</t>
+          <t>Los nombres que olvidamos</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>María Dolores Avia</t>
+          <t>María F. Fitzgerald</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -1283,12 +1279,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Los nombres que olvidamos</t>
+          <t>Solo un poco aquí</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>María F. Fitzgerald</t>
+          <t>María Ospina Pizano</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -1296,12 +1292,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Solo un poco aquí</t>
+          <t>Este es el mar</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>María Ospina Pizano</t>
+          <t>Mariana Enriquez</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -1309,12 +1305,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Este es el mar</t>
+          <t>Niñapájaroglaciar</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Mariana Enriquez</t>
+          <t>Mariana Matija</t>
         </is>
       </c>
       <c r="C67" t="inlineStr"/>
@@ -1322,12 +1318,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Niñapájaroglaciar</t>
+          <t>Mañana no te presentes</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Mariana Matija</t>
+          <t>Marta Orrantia</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -1335,12 +1331,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Mañana no te presentes</t>
+          <t>Cuentos</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Marta Orrantia</t>
+          <t>Marvel Moreno</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -1348,7 +1344,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cuentos</t>
+          <t>En diciembre llegaban las garzas</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1361,12 +1357,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>En diciembre llegaban las garzas</t>
+          <t>La casa de la belleza</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Marvel Moreno</t>
+          <t>Melba Escobar</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -1374,12 +1370,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>La casa de la belleza</t>
+          <t>Reinventar el amor</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Melba Escobar</t>
+          <t>Mona Chollet</t>
         </is>
       </c>
       <c r="C72" t="inlineStr"/>
@@ -1387,12 +1383,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Reinventar el amor</t>
+          <t>El enigma del amuleto</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Mona Chollet</t>
+          <t>Mónica Acebedo</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -1400,12 +1396,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>El enigma del amuleto</t>
+          <t>Los errantes</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Mónica Acebedo</t>
+          <t>Olga Tokarczuk</t>
         </is>
       </c>
       <c r="C74" t="inlineStr"/>
@@ -1413,12 +1409,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Los errantes</t>
+          <t>La mujer del pelo rojo</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Olga Tokarczuk</t>
+          <t>Orhan Pamuk</t>
         </is>
       </c>
       <c r="C75" t="inlineStr"/>
@@ -1426,12 +1422,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>La mujer del pelo rojo</t>
+          <t>Lo que no tiene nombre</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Orhan Pamuk</t>
+          <t>Piedad Bonnet</t>
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
@@ -1439,12 +1435,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Lo que no tiene nombre</t>
+          <t>Diccionario</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Piedad Bonnet</t>
+          <t>RAE</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -1452,12 +1448,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Diccionario</t>
+          <t>Horizontes para la paz</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>RAE</t>
+          <t>Rafael Pardo</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -1465,12 +1461,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Horizontes para la paz</t>
+          <t>Lola Vendetta: Katanazo al amor romántico</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Rafael Pardo</t>
+          <t>Raquel Riba Rossy</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -1478,12 +1474,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Lola Vendetta: Katanazo al amor romántico</t>
+          <t>Nombres y animales</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Raquel Riba Rossy</t>
+          <t>Rita Indiana</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -1491,12 +1487,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Nombres y animales</t>
+          <t>El peso del corazón</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Rita Indiana</t>
+          <t>Rosa Montero</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -1504,7 +1500,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>El peso del corazón</t>
+          <t>La ridícula idea de no volverte a ver</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1517,12 +1513,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>La ridícula idea de no volverte a ver</t>
+          <t>El crisantemo y la espada</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Rosa Montero</t>
+          <t>Ruth Benedict</t>
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
@@ -1530,12 +1526,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>El crisantemo y la espada</t>
+          <t>Pájaros en la Boca</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Ruth Benedict</t>
+          <t>Samanta Schweblin</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -1543,12 +1539,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Pájaros en la Boca</t>
+          <t>La dependienta</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Samanta Schweblin</t>
+          <t>Sayaka Murata</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -1556,12 +1552,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>La dependienta</t>
+          <t>Nada que decir</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Sayaka Murata</t>
+          <t>Silvia Hidalgo</t>
         </is>
       </c>
       <c r="C86" t="inlineStr"/>
@@ -1569,12 +1565,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Nada que decir</t>
+          <t>La campana de cristal</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Silvia Hidalgo</t>
+          <t>Silvia Plath</t>
         </is>
       </c>
       <c r="C87" t="inlineStr"/>
@@ -1582,12 +1578,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>La campana de cristal</t>
+          <t>Cauce y río</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Silvia Plath</t>
+          <t>Silvia Rivera Cusicanqui</t>
         </is>
       </c>
       <c r="C88" t="inlineStr"/>
@@ -1595,42 +1591,42 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Cauce y río</t>
+          <t>El mundo de ayer</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Silvia Rivera Cusicanqui</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr"/>
+          <t>Stefan Zweig</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>El mundo de ayer</t>
+          <t>Emily Dickinson y lo incompleto</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Stefan Zweig</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Alma</t>
-        </is>
-      </c>
+          <t>Tania Ganitsky</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Emily Dickinson y lo incompleto</t>
+          <t>The once and future king</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Tania Ganitsky</t>
+          <t>TH White</t>
         </is>
       </c>
       <c r="C91" t="inlineStr"/>
@@ -1638,12 +1634,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>The once and future king</t>
+          <t>Budismo para principiantes</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>TH White</t>
+          <t>Thubten Chodron</t>
         </is>
       </c>
       <c r="C92" t="inlineStr"/>
@@ -1651,12 +1647,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Budismo para principiantes</t>
+          <t>Cuántas veces nunca más</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Thubten Chodron</t>
+          <t>Valentina Upegui</t>
         </is>
       </c>
       <c r="C93" t="inlineStr"/>
@@ -1664,12 +1660,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Cuántas veces nunca más</t>
+          <t>Aguas de estuario</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Valentina Upegui</t>
+          <t>Velia Vidal</t>
         </is>
       </c>
       <c r="C94" t="inlineStr"/>
@@ -1677,7 +1673,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Aguas de estuario</t>
+          <t>Diez lunas para una espera</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -1690,20 +1686,24 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Diez lunas para una espera</t>
+          <t>Al faro</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Velia Vidal</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr"/>
+          <t>Virginia Woolf</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Lumen</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Al faro</t>
+          <t>El cuarto de Jacob</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -1720,7 +1720,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>El cuarto de Jacob</t>
+          <t>El lector común</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -1737,7 +1737,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>El lector común</t>
+          <t>Fin de viaje</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -1754,7 +1754,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Fin de viaje</t>
+          <t>Los años</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -1771,7 +1771,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Los años</t>
+          <t>Momentos de vida</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -1788,7 +1788,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Momentos de vida</t>
+          <t>Noche y día</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -1805,7 +1805,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Noche y día</t>
+          <t>Tres guineas</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -1822,7 +1822,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Tres guineas</t>
+          <t>Una habitación propia</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -1830,21 +1830,17 @@
           <t>Virginia Woolf</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Lumen</t>
-        </is>
-      </c>
+      <c r="C104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Una habitación propia</t>
+          <t>La casa de las bellas durmientes</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Virginia Woolf</t>
+          <t>Yasunari Kawabata</t>
         </is>
       </c>
       <c r="C105" t="inlineStr"/>
@@ -1852,7 +1848,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>La casa de las bellas durmientes</t>
+          <t>Mil grullas</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -1861,19 +1857,6 @@
         </is>
       </c>
       <c r="C106" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Mil grullas</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Yasunari Kawabata</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated book in wishlist
</commit_message>
<xml_diff>
--- a/data/nini/Wishlist.xlsx
+++ b/data/nini/Wishlist.xlsx
@@ -1157,7 +1157,11 @@
           <t>Maggie O'Farrell</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Libros del Asteroide</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">

</xml_diff>

<commit_message>
Added book to wishlist
</commit_message>
<xml_diff>
--- a/data/nini/Wishlist.xlsx
+++ b/data/nini/Wishlist.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1811,6 +1811,23 @@
       </c>
       <c r="C103" t="inlineStr"/>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momentos estelares de la humanidad </t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Stefan Zweig</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Deleted book: Orwell from Nini's wishlist
</commit_message>
<xml_diff>
--- a/data/nini/Wishlist.xlsx
+++ b/data/nini/Wishlist.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1835,15 +1835,6 @@
       <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr"/>
     </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Orwell</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr"/>
-      <c r="C106" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>